<commit_message>
feat: concluir backend node e frontend de autenticacao de funcionarios e mesas
</commit_message>
<xml_diff>
--- a/tabelas/trabalho ratatue tabelas.xlsx
+++ b/tabelas/trabalho ratatue tabelas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlos\Documents\projetofacu\ratatue\tabelas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9B4B563-E694-46C8-9AA5-223C403103CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1501391B-8F94-42C6-847A-ADF292167E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{78DECD3D-1296-4C1C-BF3B-2AB54ED1ECA8}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="31">
   <si>
     <t>Funcionarios</t>
   </si>
@@ -120,6 +120,18 @@
   </si>
   <si>
     <t>preco_unitario_pago</t>
+  </si>
+  <si>
+    <t>Funcionários: Tabela isolada (apenas para login e controle de quem acessa o quê).</t>
+  </si>
+  <si>
+    <t>Mesas ──(1 para 1 Ativo)──► Comandas: Vinculadas pelo id_mesa. Apenas uma comanda pode estar 'Aberta' por mesa por vez.</t>
+  </si>
+  <si>
+    <t>Comandas ──(1 para Muitos)──► Pedidos_Itens: Vinculadas pelo id_comanda. Uma comanda ativa recebe várias linhas de itens consumidos.</t>
+  </si>
+  <si>
+    <t>Cardapio ──(1 para Muitos)──► Pedidos_Itens: Vinculadas pelo id_produto. O cardápio fornece os preços e nomes para os itens pedidos.</t>
   </si>
 </sst>
 </file>
@@ -156,7 +168,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -164,16 +176,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -508,7 +541,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3305C810-5FCD-4EDA-9BBD-F1C6BA41BC28}">
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="33" customWidth="1"/>
@@ -622,9 +655,29 @@
         <v>20</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="E8" t="s">
         <v>21</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="63.75" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A9" s="3" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="90.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="120.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>